<commit_message>
Ajustar horarios visitas PA a 10:00, 11:00 y 12:00
Co-authored-by: anibaloperacionesWes <anibaloperacionesWes@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/reports/Corporación_Puente_Alto/visitas/Visitas_colegios_Puente_Alto_2026-10-14.xlsx
+++ b/reports/Corporación_Puente_Alto/visitas/Visitas_colegios_Puente_Alto_2026-10-14.xlsx
@@ -517,7 +517,7 @@
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>11:00</t>
         </is>
       </c>
     </row>
@@ -534,7 +534,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>12:00</t>
         </is>
       </c>
     </row>

</xml_diff>